<commit_message>
feat(compras): implementa painel de panorama global de compras por fornecedor e exclusao da lista
</commit_message>
<xml_diff>
--- a/public/templates/modelo_cotacao.xlsx
+++ b/public/templates/modelo_cotacao.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ander\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3712DB62-E3BB-4B4C-A004-1C86594184E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{2D68E6E1-AF02-456C-A52D-1D93AEDB993F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="16">
   <si>
     <t>FORÇA MÁXIMA VEDAÇÕES - SOLICITAÇÃO DE COTAÇÃO</t>
   </si>
@@ -61,6 +61,24 @@
     <t>Qtd</t>
   </si>
   <si>
+    <t>Frete</t>
+  </si>
+  <si>
+    <t>Preço Unit. (R$)</t>
+  </si>
+  <si>
+    <t>Preço Total</t>
+  </si>
+  <si>
+    <t>Imposto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Preço Unit Referencia </t>
+  </si>
+  <si>
+    <t>Fornecedor</t>
+  </si>
+  <si>
     <t>W25000500</t>
   </si>
   <si>
@@ -68,24 +86,6 @@
   </si>
   <si>
     <t xml:space="preserve"> 127.00X12.70X3.17</t>
-  </si>
-  <si>
-    <t>Frete</t>
-  </si>
-  <si>
-    <t>Preço Unit. (R$)</t>
-  </si>
-  <si>
-    <t>Preço Total</t>
-  </si>
-  <si>
-    <t>Imposto</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Preço Unit Referencia </t>
-  </si>
-  <si>
-    <t>Fornecedor</t>
   </si>
   <si>
     <t>SKS</t>
@@ -712,89 +712,49 @@
       <c r="A10" s="1">
         <v>1</v>
       </c>
-      <c r="B10" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E10" s="2">
-        <v>5</v>
-      </c>
+      <c r="B10" s="3"/>
+      <c r="C10" s="3"/>
+      <c r="D10" s="3"/>
+      <c r="E10" s="2"/>
       <c r="F10" s="10"/>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="1">
         <v>2</v>
       </c>
-      <c r="B11" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E11" s="2">
-        <v>5</v>
-      </c>
+      <c r="B11" s="3"/>
+      <c r="C11" s="3"/>
+      <c r="D11" s="3"/>
+      <c r="E11" s="2"/>
       <c r="F11" s="10"/>
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="1">
         <v>3</v>
       </c>
-      <c r="B12" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E12" s="2">
-        <v>1</v>
-      </c>
+      <c r="B12" s="3"/>
+      <c r="C12" s="3"/>
+      <c r="D12" s="3"/>
+      <c r="E12" s="2"/>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" s="2">
         <v>4</v>
       </c>
-      <c r="B13" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D13" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E13" s="2">
-        <v>1</v>
-      </c>
+      <c r="B13" s="3"/>
+      <c r="C13" s="3"/>
+      <c r="D13" s="3"/>
+      <c r="E13" s="2"/>
       <c r="F13" s="10"/>
     </row>
     <row r="14" spans="1:6">
       <c r="A14" s="2">
         <v>5</v>
       </c>
-      <c r="B14" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D14" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E14" s="2">
-        <v>4</v>
-      </c>
+      <c r="B14" s="3"/>
+      <c r="C14" s="3"/>
+      <c r="D14" s="3"/>
+      <c r="E14" s="2"/>
       <c r="F14" s="10"/>
     </row>
     <row r="15" spans="1:6">
@@ -969,7 +929,7 @@
       <c r="G7" s="7"/>
       <c r="H7" s="7"/>
       <c r="I7" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="8" spans="1:10">
@@ -999,19 +959,19 @@
         <v>5</v>
       </c>
       <c r="F9" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="H9" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="I9" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="G9" s="6" t="s">
+      <c r="J9" s="9" t="s">
         <v>11</v>
-      </c>
-      <c r="H9" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="I9" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="J9" s="9" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="10" spans="1:10">
@@ -1019,13 +979,13 @@
         <v>1</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="E10" s="2">
         <v>5</v>

</xml_diff>

<commit_message>
fix(excel): use protocol ID for excel export filename to prevent generic repetition
</commit_message>
<xml_diff>
--- a/public/templates/modelo_cotacao.xlsx
+++ b/public/templates/modelo_cotacao.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ander\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2D68E6E1-AF02-456C-A52D-1D93AEDB993F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A025839D-6EE9-4264-95C5-8A53CB1C78D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -99,7 +99,7 @@
     <numFmt numFmtId="44" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="&quot;R$&quot;\ #,##0.00"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -135,6 +135,14 @@
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -222,7 +230,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -249,6 +257,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="2">
@@ -679,17 +688,17 @@
       <c r="A7" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="B7" s="12"/>
-      <c r="C7" s="12"/>
-      <c r="D7" s="12"/>
-      <c r="E7" s="12"/>
+      <c r="B7" s="13"/>
+      <c r="C7" s="13"/>
+      <c r="D7" s="13"/>
+      <c r="E7" s="13"/>
     </row>
     <row r="8" spans="1:6">
-      <c r="A8" s="12"/>
-      <c r="B8" s="12"/>
-      <c r="C8" s="12"/>
-      <c r="D8" s="12"/>
-      <c r="E8" s="12"/>
+      <c r="A8" s="13"/>
+      <c r="B8" s="13"/>
+      <c r="C8" s="13"/>
+      <c r="D8" s="13"/>
+      <c r="E8" s="13"/>
     </row>
     <row r="9" spans="1:6" ht="40.15" customHeight="1">
       <c r="A9" s="6" t="s">
@@ -709,9 +718,7 @@
       </c>
     </row>
     <row r="10" spans="1:6">
-      <c r="A10" s="1">
-        <v>1</v>
-      </c>
+      <c r="A10" s="1"/>
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
       <c r="D10" s="3"/>
@@ -719,9 +726,7 @@
       <c r="F10" s="10"/>
     </row>
     <row r="11" spans="1:6">
-      <c r="A11" s="1">
-        <v>2</v>
-      </c>
+      <c r="A11" s="1"/>
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
       <c r="D11" s="3"/>
@@ -729,18 +734,14 @@
       <c r="F11" s="10"/>
     </row>
     <row r="12" spans="1:6">
-      <c r="A12" s="1">
-        <v>3</v>
-      </c>
+      <c r="A12" s="1"/>
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
       <c r="D12" s="3"/>
       <c r="E12" s="2"/>
     </row>
     <row r="13" spans="1:6">
-      <c r="A13" s="2">
-        <v>4</v>
-      </c>
+      <c r="A13" s="2"/>
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
       <c r="D13" s="3"/>
@@ -748,9 +749,7 @@
       <c r="F13" s="10"/>
     </row>
     <row r="14" spans="1:6">
-      <c r="A14" s="2">
-        <v>5</v>
-      </c>
+      <c r="A14" s="2"/>
       <c r="B14" s="3"/>
       <c r="C14" s="3"/>
       <c r="D14" s="3"/>
@@ -758,135 +757,105 @@
       <c r="F14" s="10"/>
     </row>
     <row r="15" spans="1:6">
-      <c r="A15" s="2">
-        <v>6</v>
-      </c>
+      <c r="A15" s="2"/>
       <c r="B15" s="3"/>
       <c r="C15" s="3"/>
       <c r="D15" s="3"/>
       <c r="E15" s="2"/>
     </row>
     <row r="16" spans="1:6">
-      <c r="A16" s="2">
-        <v>7</v>
-      </c>
+      <c r="A16" s="2"/>
       <c r="B16" s="3"/>
       <c r="C16" s="3"/>
       <c r="D16" s="3"/>
       <c r="E16" s="2"/>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" s="2">
-        <v>8</v>
-      </c>
+      <c r="A17" s="2"/>
       <c r="B17" s="3"/>
       <c r="C17" s="3"/>
       <c r="D17" s="3"/>
       <c r="E17" s="3"/>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="2">
-        <v>9</v>
-      </c>
+      <c r="A18" s="2"/>
       <c r="B18" s="3"/>
       <c r="C18" s="3"/>
       <c r="D18" s="3"/>
       <c r="E18" s="3"/>
     </row>
-    <row r="19" spans="1:5">
-      <c r="A19" s="2">
-        <v>10</v>
-      </c>
+    <row r="19" spans="1:5" ht="15">
+      <c r="A19" s="2"/>
       <c r="B19" s="3"/>
       <c r="C19" s="3"/>
       <c r="D19" s="3"/>
-      <c r="E19" s="3"/>
+      <c r="E19" s="12"/>
     </row>
     <row r="20" spans="1:5">
-      <c r="A20" s="2">
-        <v>11</v>
-      </c>
+      <c r="A20" s="2"/>
       <c r="B20" s="3"/>
       <c r="C20" s="3"/>
       <c r="D20" s="3"/>
       <c r="E20" s="3"/>
     </row>
     <row r="21" spans="1:5">
-      <c r="A21" s="2">
-        <v>12</v>
-      </c>
+      <c r="A21" s="2"/>
       <c r="B21" s="3"/>
       <c r="C21" s="3"/>
       <c r="D21" s="3"/>
       <c r="E21" s="3"/>
     </row>
     <row r="22" spans="1:5">
-      <c r="A22" s="2">
-        <v>13</v>
-      </c>
+      <c r="A22" s="2"/>
       <c r="B22" s="3"/>
       <c r="C22" s="3"/>
       <c r="D22" s="3"/>
       <c r="E22" s="3"/>
     </row>
     <row r="23" spans="1:5">
-      <c r="A23" s="2">
-        <v>14</v>
-      </c>
+      <c r="A23" s="2"/>
       <c r="B23" s="3"/>
       <c r="C23" s="3"/>
       <c r="D23" s="3"/>
       <c r="E23" s="3"/>
     </row>
     <row r="24" spans="1:5">
-      <c r="A24" s="2">
-        <v>15</v>
-      </c>
+      <c r="A24" s="2"/>
       <c r="B24" s="3"/>
       <c r="C24" s="3"/>
       <c r="D24" s="3"/>
       <c r="E24" s="3"/>
     </row>
     <row r="25" spans="1:5">
-      <c r="A25" s="2">
-        <v>16</v>
-      </c>
+      <c r="A25" s="2"/>
       <c r="B25" s="3"/>
       <c r="C25" s="3"/>
       <c r="D25" s="3"/>
       <c r="E25" s="3"/>
     </row>
     <row r="26" spans="1:5">
-      <c r="A26" s="2">
-        <v>17</v>
-      </c>
+      <c r="A26" s="2"/>
       <c r="B26" s="3"/>
       <c r="C26" s="3"/>
       <c r="D26" s="3"/>
       <c r="E26" s="3"/>
     </row>
     <row r="27" spans="1:5">
-      <c r="A27" s="2">
-        <v>18</v>
-      </c>
+      <c r="A27" s="2"/>
       <c r="B27" s="3"/>
       <c r="C27" s="3"/>
       <c r="D27" s="3"/>
       <c r="E27" s="3"/>
     </row>
     <row r="28" spans="1:5">
-      <c r="A28" s="2">
-        <v>19</v>
-      </c>
+      <c r="A28" s="2"/>
       <c r="B28" s="3"/>
       <c r="C28" s="3"/>
       <c r="D28" s="3"/>
       <c r="E28" s="3"/>
     </row>
     <row r="29" spans="1:5">
-      <c r="A29" s="2">
-        <v>20</v>
-      </c>
+      <c r="A29" s="2"/>
       <c r="B29" s="3"/>
       <c r="C29" s="3"/>
       <c r="D29" s="3"/>
@@ -921,11 +890,11 @@
       <c r="A7" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="B7" s="12"/>
-      <c r="C7" s="12"/>
-      <c r="D7" s="12"/>
-      <c r="E7" s="12"/>
-      <c r="F7" s="12"/>
+      <c r="B7" s="13"/>
+      <c r="C7" s="13"/>
+      <c r="D7" s="13"/>
+      <c r="E7" s="13"/>
+      <c r="F7" s="13"/>
       <c r="G7" s="7"/>
       <c r="H7" s="7"/>
       <c r="I7" t="s">
@@ -933,12 +902,12 @@
       </c>
     </row>
     <row r="8" spans="1:10">
-      <c r="A8" s="12"/>
-      <c r="B8" s="12"/>
-      <c r="C8" s="12"/>
-      <c r="D8" s="12"/>
-      <c r="E8" s="12"/>
-      <c r="F8" s="12"/>
+      <c r="A8" s="13"/>
+      <c r="B8" s="13"/>
+      <c r="C8" s="13"/>
+      <c r="D8" s="13"/>
+      <c r="E8" s="13"/>
+      <c r="F8" s="13"/>
       <c r="G8" s="7"/>
       <c r="H8" s="7"/>
     </row>

</xml_diff>